<commit_message>
Update Levantamento de correspondencia CIATA x CNEFE.xlsx
</commit_message>
<xml_diff>
--- a/Levantamento de correspondencia CIATA x CNEFE.xlsx
+++ b/Levantamento de correspondencia CIATA x CNEFE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f6f68d678cfe6957/Documentos/Mestrado/TCC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{85E78417-1F04-4D53-95B5-9BFF93B0B7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="8_{85E78417-1F04-4D53-95B5-9BFF93B0B7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72F1F076-9EF9-4BCD-B599-14CD42EC04B7}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-3540" windowWidth="29040" windowHeight="15840" xr2:uid="{75E32A08-3FBA-4F92-879D-79AC4B6A16E5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
   <si>
     <t>CI_</t>
   </si>
@@ -99,6 +99,81 @@
   </si>
   <si>
     <t>NÃO EXISTIA EM 2022 (Coleta CNEFE)</t>
+  </si>
+  <si>
+    <t>RUA GENTIL ALCHIERI</t>
+  </si>
+  <si>
+    <t>RUA DORVAL BENATTI</t>
+  </si>
+  <si>
+    <t>RUA VILMAR BERFT</t>
+  </si>
+  <si>
+    <t>RUA CEREJEIRA</t>
+  </si>
+  <si>
+    <t>RUA GUAJUVIRA</t>
+  </si>
+  <si>
+    <t>AVENIDA MAUA</t>
+  </si>
+  <si>
+    <t>RUA REINALDO LINDEN</t>
+  </si>
+  <si>
+    <t>RUA DAS PEROBAS</t>
+  </si>
+  <si>
+    <t>AVENIDA DAS FLORES</t>
+  </si>
+  <si>
+    <t>RUA HERMINIA BARBIERI BIGATON</t>
+  </si>
+  <si>
+    <t>AVENIDA ATAIDE ROBERTO ESCHER</t>
+  </si>
+  <si>
+    <t>RUA GOIABEIRAS</t>
+  </si>
+  <si>
+    <t>RUA DA GOIABEIRA</t>
+  </si>
+  <si>
+    <t>RUA CEDRO</t>
+  </si>
+  <si>
+    <t>RUA CARLOS MAGRO</t>
+  </si>
+  <si>
+    <t>RUA LOURO BRANCO</t>
+  </si>
+  <si>
+    <t>RUA CAMELIA</t>
+  </si>
+  <si>
+    <t>RUA VALDI BERFT 2 PARTE</t>
+  </si>
+  <si>
+    <t>RUA VALDIR BERFT</t>
+  </si>
+  <si>
+    <t>RUA ERNESTO LORENZETI</t>
+  </si>
+  <si>
+    <t>RUA ANTONIO LORENZETTI</t>
+  </si>
+  <si>
+    <t>RUA PITANGUEIRA</t>
+  </si>
+  <si>
+    <t>RUA DELMAR SEVERO</t>
+  </si>
+  <si>
+    <t>RUA EUGENIO RAVACHE</t>
+  </si>
+  <si>
+    <t>AV. ATAIDES ROBERTO ESCHER</t>
   </si>
 </sst>
 </file>
@@ -173,9 +248,6 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -184,6 +256,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88B9B46C-FB57-4C40-89C6-D97D7C885C05}">
-  <dimension ref="A2:F27"/>
+  <dimension ref="B2:J30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="40" customWidth="1"/>
@@ -527,37 +602,47 @@
     <col min="5" max="5" width="17.42578125" customWidth="1"/>
     <col min="6" max="6" width="40.140625" customWidth="1"/>
     <col min="7" max="7" width="33" customWidth="1"/>
+    <col min="8" max="8" width="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="40.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1" t="s">
+    <row r="2" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="2" t="s">
+      <c r="E2" s="6"/>
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
+      <c r="H3" s="3"/>
+      <c r="I3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C4">
@@ -572,8 +657,17 @@
       <c r="F4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H4" s="3">
+        <v>1</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>7</v>
       </c>
@@ -589,22 +683,40 @@
       <c r="F5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H5" s="3">
+        <v>2</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>9</v>
       </c>
       <c r="C6">
         <v>39</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H6" s="3">
+        <v>3</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>11</v>
       </c>
@@ -617,8 +729,17 @@
       <c r="E7">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H7" s="3">
+        <v>4</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -631,8 +752,17 @@
       <c r="E8">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H8" s="3">
+        <v>5</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>15</v>
       </c>
@@ -645,80 +775,308 @@
       <c r="E9">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
-      <c r="B21" s="5" t="s">
+      <c r="H9" s="3">
+        <v>6</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11">
+        <v>33</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16">
+        <v>29</v>
+      </c>
+      <c r="D16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17">
+        <v>29</v>
+      </c>
+      <c r="D17" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18">
+        <v>26</v>
+      </c>
+      <c r="D18" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20">
+        <v>21</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21">
+        <v>21</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22">
+        <v>20</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23">
+        <v>18</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24">
+        <v>18</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25">
         <v>17</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="4">
-        <v>1</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="4">
-        <v>2</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="4">
-        <v>3</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="4">
-        <v>4</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="4">
-        <v>5</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
-        <v>6</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>20</v>
+      <c r="D25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26">
+        <v>16</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27">
+        <v>16</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28">
+        <v>16</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29">
+        <v>14</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>44</v>
+      </c>
+      <c r="C30">
+        <v>13</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Visualização de Quadras CI
</commit_message>
<xml_diff>
--- a/Levantamento de correspondencia CIATA x CNEFE.xlsx
+++ b/Levantamento de correspondencia CIATA x CNEFE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f6f68d678cfe6957/Documentos/Mestrado/TCC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="8_{85E78417-1F04-4D53-95B5-9BFF93B0B7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72F1F076-9EF9-4BCD-B599-14CD42EC04B7}"/>
+  <xr:revisionPtr revIDLastSave="102" documentId="8_{85E78417-1F04-4D53-95B5-9BFF93B0B7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D0DE366-92A7-494E-8061-989616E68E0A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-3540" windowWidth="29040" windowHeight="15840" xr2:uid="{75E32A08-3FBA-4F92-879D-79AC4B6A16E5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="47">
   <si>
     <t>CI_</t>
   </si>
@@ -174,13 +174,16 @@
   </si>
   <si>
     <t>AV. ATAIDES ROBERTO ESCHER</t>
+  </si>
+  <si>
+    <t>NÃO EXISTE NO MAPS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,6 +209,20 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -246,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -260,6 +277,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -275,6 +297,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -642,19 +668,19 @@
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="9">
         <v>82</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="9">
         <v>81</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="9" t="s">
         <v>4</v>
       </c>
       <c r="H4" s="3">
@@ -668,19 +694,19 @@
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="B5" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="9">
         <v>237</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="9">
         <v>169</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="9" t="s">
         <v>8</v>
       </c>
       <c r="H5" s="3">
@@ -694,16 +720,17 @@
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+      <c r="B6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="9">
         <v>39</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="E6" s="9"/>
+      <c r="F6" s="8" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="3">
@@ -717,17 +744,18 @@
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7">
-        <v>34</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7">
-        <v>3</v>
+      <c r="B7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="9">
+        <v>21</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="H7" s="3">
         <v>4</v>
@@ -740,17 +768,18 @@
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8">
-        <v>2</v>
+      <c r="B8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="9">
+        <v>21</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="F8" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="H8" s="3">
         <v>5</v>
@@ -763,17 +792,18 @@
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9">
-        <v>34</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
+      <c r="B9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="9">
+        <v>16</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="H9" s="3">
         <v>6</v>
@@ -786,53 +816,54 @@
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10">
-        <v>33</v>
-      </c>
-      <c r="D10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
+      <c r="B10" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="9">
+        <v>16</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="8" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C11">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C12">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="2" t="s">
-        <v>24</v>
+      <c r="B13" t="s">
+        <v>15</v>
       </c>
       <c r="C13">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
         <v>16</v>
@@ -842,11 +873,11 @@
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
-        <v>25</v>
+      <c r="B14" t="s">
+        <v>21</v>
       </c>
       <c r="C14">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
@@ -857,10 +888,10 @@
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C15">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
         <v>16</v>
@@ -870,11 +901,11 @@
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
-        <v>27</v>
+      <c r="B16" t="s">
+        <v>23</v>
       </c>
       <c r="C16">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D16" t="s">
         <v>16</v>
@@ -885,10 +916,10 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C17">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D17" t="s">
         <v>16</v>
@@ -898,69 +929,72 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>29</v>
+      <c r="B18" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="C18">
+        <v>30</v>
+      </c>
+      <c r="D18" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D18" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="7">
         <v>30</v>
       </c>
-      <c r="C19">
-        <v>24</v>
-      </c>
-      <c r="D19" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19">
-        <v>0</v>
+      <c r="D19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="7">
+        <v>0</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="C20">
-        <v>21</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
+      </c>
+      <c r="D20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C21">
-        <v>21</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
+      </c>
+      <c r="D21" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>34</v>
+      <c r="B22" t="s">
+        <v>29</v>
       </c>
       <c r="C22">
-        <v>20</v>
-      </c>
-      <c r="D22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" t="s">
         <v>16</v>
       </c>
       <c r="E22">
@@ -969,12 +1003,12 @@
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C23">
-        <v>18</v>
-      </c>
-      <c r="D23" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" t="s">
         <v>16</v>
       </c>
       <c r="E23">
@@ -982,11 +1016,11 @@
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>36</v>
+      <c r="B24" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="C24">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>16</v>
@@ -997,10 +1031,10 @@
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C25">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>16</v>
@@ -1011,30 +1045,30 @@
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C26">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>39</v>
+        <v>16</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C27">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>41</v>
+        <v>16</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">

</xml_diff>